<commit_message>
edit data in portfolio_aom.xlsx
</commit_message>
<xml_diff>
--- a/portfolio_aom.xlsx
+++ b/portfolio_aom.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\StockInvestment\StockInvestment\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\StockInvestment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{310C03C2-6A1C-481F-8EA5-4E07BE67A871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF57E77-1815-46BC-B3BD-8157DD015088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4260" yWindow="4635" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -443,9 +443,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -467,7 +467,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
@@ -478,7 +478,7 @@
         <v>6.19</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -489,18 +489,18 @@
         <v>20.98</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B5">
+        <v>300</v>
+      </c>
+      <c r="C5">
         <v>57.68</v>
       </c>
-      <c r="C5">
-        <v>45.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
@@ -511,7 +511,7 @@
         <v>39.619999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -522,7 +522,7 @@
         <v>23.05</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -533,7 +533,7 @@
         <v>32.799999999999997</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
@@ -544,7 +544,7 @@
         <v>10.220000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
@@ -555,7 +555,7 @@
         <v>7.26</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
@@ -566,7 +566,7 @@
         <v>21.73</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -577,7 +577,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
@@ -588,7 +588,7 @@
         <v>18.760000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>6</v>
       </c>
@@ -599,7 +599,7 @@
         <v>28.87</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
@@ -610,49 +610,49 @@
         <v>10.42</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
     </row>
   </sheetData>

</xml_diff>